<commit_message>
Final fix: Robust Excel parsing and time refresh
- Enhanced Excel parsing with robust type conversion and error tolerance
- Automatic skip invalid rows instead of failing entire file
- Support various number formats (commas, currency symbols)
- Auto trim whitespace from text fields
- Force refresh results after calculation with timestamp
- Auto navigate to results page after successful calculation
- Clear old results before saving new ones
- Display last update time on results page

🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/salaries.xlsx
+++ b/salaries.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="25600" windowHeight="12080"/>
+    <workbookView windowWidth="23152" windowHeight="11055"/>
   </bookViews>
   <sheets>
     <sheet name="salaries" sheetId="1" r:id="rId1"/>
@@ -681,12 +681,9 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1223,30 +1220,30 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:E37"/>
-  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14" outlineLevelCol="4"/>
+  <sheetFormatPr defaultColWidth="8.72566371681416" defaultRowHeight="13.5" outlineLevelCol="4"/>
   <cols>
-    <col min="1" max="1" width="8.72727272727273" style="1"/>
-    <col min="2" max="2" width="19.0909090909091" style="2" customWidth="1"/>
-    <col min="3" max="3" width="26.0909090909091" style="2" customWidth="1"/>
-    <col min="4" max="4" width="14.7272727272727" style="2" customWidth="1"/>
-    <col min="5" max="5" width="23.5454545454545" style="2" customWidth="1"/>
-    <col min="6" max="6" width="26.0909090909091" customWidth="1"/>
+    <col min="1" max="1" width="8.72566371681416" style="1"/>
+    <col min="2" max="2" width="19.0884955752212" style="1" customWidth="1"/>
+    <col min="3" max="3" width="26.0884955752212" style="1" customWidth="1"/>
+    <col min="4" max="4" width="14.7256637168142" style="1" customWidth="1"/>
+    <col min="5" max="5" width="23.5486725663717" style="1" customWidth="1"/>
+    <col min="6" max="6" width="26.0884955752212" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1254,152 +1251,152 @@
       <c r="A2" s="1">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="1">
         <v>202401</v>
       </c>
-      <c r="E2" s="2">
-        <v>30000</v>
+      <c r="E2" s="1">
+        <v>32000</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="1">
         <v>2</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="1">
         <v>202402</v>
       </c>
-      <c r="E3" s="2">
-        <v>29000</v>
+      <c r="E3" s="1">
+        <v>29045</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1">
         <v>3</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="1">
         <v>202403</v>
       </c>
-      <c r="E4" s="2">
-        <v>31000</v>
+      <c r="E4" s="1">
+        <v>29046</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="1">
         <v>4</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D5" s="1">
         <v>202404</v>
       </c>
-      <c r="E5" s="2">
-        <v>30000</v>
+      <c r="E5" s="1">
+        <v>29047</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="1">
         <v>5</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D6" s="1">
         <v>202405</v>
       </c>
-      <c r="E6" s="2">
-        <v>29000</v>
+      <c r="E6" s="1">
+        <v>29048</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="1">
         <v>6</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D7" s="1">
         <v>202406</v>
       </c>
-      <c r="E7" s="2">
-        <v>31000</v>
+      <c r="E7" s="1">
+        <v>29049</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="1">
         <v>7</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="1">
         <v>202407</v>
       </c>
-      <c r="E8" s="2">
-        <v>30000</v>
+      <c r="E8" s="1">
+        <v>29050</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="1">
         <v>8</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D9" s="2">
+      <c r="D9" s="1">
         <v>202408</v>
       </c>
-      <c r="E9" s="2">
-        <v>29000</v>
+      <c r="E9" s="1">
+        <v>29051</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="1">
         <v>9</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D10" s="2">
+      <c r="D10" s="1">
         <v>202409</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>31000</v>
       </c>
     </row>
@@ -1407,16 +1404,16 @@
       <c r="A11" s="1">
         <v>10</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D11" s="2">
+      <c r="D11" s="1">
         <v>202410</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>30000</v>
       </c>
     </row>
@@ -1424,16 +1421,16 @@
       <c r="A12" s="1">
         <v>11</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D12" s="2">
+      <c r="D12" s="1">
         <v>202411</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>29000</v>
       </c>
     </row>
@@ -1441,339 +1438,339 @@
       <c r="A13" s="1">
         <v>12</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C13" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D13" s="2">
+      <c r="D13" s="1">
         <v>202412</v>
       </c>
-      <c r="E13" s="2">
-        <v>31000</v>
+      <c r="E13" s="1">
+        <v>29001</v>
       </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="1">
         <v>13</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C14" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D14" s="2">
+      <c r="D14" s="1">
         <v>202401</v>
       </c>
-      <c r="E14" s="2">
-        <v>15000</v>
+      <c r="E14" s="1">
+        <v>29002</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="1">
         <v>14</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="C15" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D15" s="2">
+      <c r="D15" s="1">
         <v>202402</v>
       </c>
-      <c r="E15" s="2">
-        <v>14000</v>
+      <c r="E15" s="1">
+        <v>29003</v>
       </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="1">
         <v>15</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C16" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D16" s="2">
+      <c r="D16" s="1">
         <v>202403</v>
       </c>
-      <c r="E16" s="2">
-        <v>16000</v>
+      <c r="E16" s="1">
+        <v>29004</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="1">
         <v>16</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="C17" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D17" s="2">
+      <c r="D17" s="1">
         <v>202404</v>
       </c>
-      <c r="E17" s="2">
-        <v>15000</v>
+      <c r="E17" s="1">
+        <v>29005</v>
       </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" s="1">
         <v>17</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="C18" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D18" s="2">
+      <c r="D18" s="1">
         <v>202405</v>
       </c>
-      <c r="E18" s="2">
-        <v>14000</v>
+      <c r="E18" s="1">
+        <v>29006</v>
       </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="1">
         <v>18</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="C19" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D19" s="2">
+      <c r="D19" s="1">
         <v>202406</v>
       </c>
-      <c r="E19" s="2">
-        <v>16000</v>
+      <c r="E19" s="1">
+        <v>29007</v>
       </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="1">
         <v>19</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="B20" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="C20" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D20" s="2">
+      <c r="D20" s="1">
         <v>202407</v>
       </c>
-      <c r="E20" s="2">
-        <v>15000</v>
+      <c r="E20" s="1">
+        <v>29008</v>
       </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="1">
         <v>20</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="C21" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D21" s="2">
+      <c r="D21" s="1">
         <v>202408</v>
       </c>
-      <c r="E21" s="2">
-        <v>14000</v>
+      <c r="E21" s="1">
+        <v>29009</v>
       </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="1">
         <v>21</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="C22" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D22" s="2">
+      <c r="D22" s="1">
         <v>202409</v>
       </c>
-      <c r="E22" s="2">
-        <v>16000</v>
+      <c r="E22" s="1">
+        <v>29010</v>
       </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="1">
         <v>22</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="B23" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="C23" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D23" s="2">
+      <c r="D23" s="1">
         <v>202410</v>
       </c>
-      <c r="E23" s="2">
-        <v>15000</v>
+      <c r="E23" s="1">
+        <v>29011</v>
       </c>
     </row>
     <row r="24" spans="1:5">
       <c r="A24" s="1">
         <v>23</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="B24" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="C24" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D24" s="2">
+      <c r="D24" s="1">
         <v>202411</v>
       </c>
-      <c r="E24" s="2">
-        <v>14000</v>
+      <c r="E24" s="1">
+        <v>29012</v>
       </c>
     </row>
     <row r="25" spans="1:5">
       <c r="A25" s="1">
         <v>24</v>
       </c>
-      <c r="B25" s="4" t="s">
+      <c r="B25" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C25" s="2" t="s">
+      <c r="C25" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D25" s="2">
+      <c r="D25" s="1">
         <v>202412</v>
       </c>
-      <c r="E25" s="2">
-        <v>16000</v>
+      <c r="E25" s="1">
+        <v>29013</v>
       </c>
     </row>
     <row r="26" spans="1:5">
       <c r="A26" s="1">
         <v>25</v>
       </c>
-      <c r="B26" s="4" t="s">
+      <c r="B26" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="C26" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D26" s="2">
+      <c r="D26" s="1">
         <v>202401</v>
       </c>
-      <c r="E26" s="2">
-        <v>4000</v>
+      <c r="E26" s="1">
+        <v>29014</v>
       </c>
     </row>
     <row r="27" spans="1:5">
       <c r="A27" s="1">
         <v>26</v>
       </c>
-      <c r="B27" s="4" t="s">
+      <c r="B27" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="C27" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D27" s="2">
+      <c r="D27" s="1">
         <v>202402</v>
       </c>
-      <c r="E27" s="2">
-        <v>3900</v>
+      <c r="E27" s="1">
+        <v>29015</v>
       </c>
     </row>
     <row r="28" spans="1:5">
       <c r="A28" s="1">
         <v>27</v>
       </c>
-      <c r="B28" s="4" t="s">
+      <c r="B28" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C28" s="2" t="s">
+      <c r="C28" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D28" s="2">
+      <c r="D28" s="1">
         <v>202403</v>
       </c>
-      <c r="E28" s="2">
-        <v>4100</v>
+      <c r="E28" s="1">
+        <v>29016</v>
       </c>
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="1">
         <v>28</v>
       </c>
-      <c r="B29" s="4" t="s">
+      <c r="B29" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C29" s="2" t="s">
+      <c r="C29" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D29" s="2">
+      <c r="D29" s="1">
         <v>202404</v>
       </c>
-      <c r="E29" s="2">
-        <v>4000</v>
+      <c r="E29" s="1">
+        <v>29017</v>
       </c>
     </row>
     <row r="30" spans="1:5">
       <c r="A30" s="1">
         <v>29</v>
       </c>
-      <c r="B30" s="4" t="s">
+      <c r="B30" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C30" s="2" t="s">
+      <c r="C30" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D30" s="2">
+      <c r="D30" s="1">
         <v>202405</v>
       </c>
-      <c r="E30" s="2">
-        <v>3900</v>
+      <c r="E30" s="1">
+        <v>29018</v>
       </c>
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="1">
         <v>30</v>
       </c>
-      <c r="B31" s="4" t="s">
+      <c r="B31" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C31" s="2" t="s">
+      <c r="C31" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D31" s="2">
+      <c r="D31" s="1">
         <v>202406</v>
       </c>
-      <c r="E31" s="2">
-        <v>4100</v>
+      <c r="E31" s="1">
+        <v>29019</v>
       </c>
     </row>
     <row r="32" spans="1:5">
       <c r="A32" s="1">
         <v>31</v>
       </c>
-      <c r="B32" s="4" t="s">
+      <c r="B32" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C32" s="2" t="s">
+      <c r="C32" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D32" s="2">
+      <c r="D32" s="1">
         <v>202407</v>
       </c>
-      <c r="E32" s="2">
+      <c r="E32" s="1">
         <v>4000</v>
       </c>
     </row>
@@ -1781,16 +1778,16 @@
       <c r="A33" s="1">
         <v>32</v>
       </c>
-      <c r="B33" s="4" t="s">
+      <c r="B33" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C33" s="2" t="s">
+      <c r="C33" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D33" s="2">
+      <c r="D33" s="1">
         <v>202408</v>
       </c>
-      <c r="E33" s="2">
+      <c r="E33" s="1">
         <v>3900</v>
       </c>
     </row>
@@ -1798,16 +1795,16 @@
       <c r="A34" s="1">
         <v>33</v>
       </c>
-      <c r="B34" s="4" t="s">
+      <c r="B34" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C34" s="2" t="s">
+      <c r="C34" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D34" s="2">
+      <c r="D34" s="1">
         <v>202409</v>
       </c>
-      <c r="E34" s="2">
+      <c r="E34" s="1">
         <v>4100</v>
       </c>
     </row>
@@ -1815,16 +1812,16 @@
       <c r="A35" s="1">
         <v>34</v>
       </c>
-      <c r="B35" s="4" t="s">
+      <c r="B35" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C35" s="2" t="s">
+      <c r="C35" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D35" s="2">
+      <c r="D35" s="1">
         <v>202410</v>
       </c>
-      <c r="E35" s="2">
+      <c r="E35" s="1">
         <v>4000</v>
       </c>
     </row>
@@ -1832,16 +1829,16 @@
       <c r="A36" s="1">
         <v>35</v>
       </c>
-      <c r="B36" s="4" t="s">
+      <c r="B36" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C36" s="2" t="s">
+      <c r="C36" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D36" s="2">
+      <c r="D36" s="1">
         <v>202411</v>
       </c>
-      <c r="E36" s="2">
+      <c r="E36" s="1">
         <v>3900</v>
       </c>
     </row>
@@ -1849,16 +1846,16 @@
       <c r="A37" s="1">
         <v>36</v>
       </c>
-      <c r="B37" s="4" t="s">
+      <c r="B37" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C37" s="2" t="s">
+      <c r="C37" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D37" s="2">
+      <c r="D37" s="1">
         <v>202412</v>
       </c>
-      <c r="E37" s="2">
+      <c r="E37" s="1">
         <v>4100</v>
       </c>
     </row>

</xml_diff>